<commit_message>
Excel: Folgeperiode beginnt 01.08.2026, Beltz unverändert
Neuer Stichtag 5; Folgeperiode nutzt Stand 4 (01.08.2026) bis Stand 5.
Die Berechnung ohne Kaltwasser gilt erst ab August 2026, Beltz bleibt
bis 19.06.2026 wie bisher.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WieYhBz7P2F1oyihzgkzQY
</commit_message>
<xml_diff>
--- a/NK_Abrechnung_Excel.xlsx
+++ b/NK_Abrechnung_Excel.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="257">
   <si>
     <t xml:space="preserve">NK-Abrechnung Teinacher Str. 4 – Excel-Version</t>
   </si>
@@ -57,7 +57,7 @@
     <t xml:space="preserve">Übersicht – Ergebnisse je Partei und Vergleich mit den dokumentierten Werten (Kontrolle).</t>
   </si>
   <si>
-    <t xml:space="preserve">Zählerstände – Ablesedatum und Zählerstand je Stichtag (Stand 4 = Folgeperiode, noch leer).</t>
+    <t xml:space="preserve">Zählerstände – Ablesedatum und Zählerstand je Stichtag (Stand 4 = 01.08.2026 Start Folgeperiode, Stand 5 = Ende, noch leer).</t>
   </si>
   <si>
     <t xml:space="preserve">Kosten – Strompreis, Grundpreis, Wasser-/Niederschlagstarife, Versicherung, Grundsteuer.</t>
@@ -75,13 +75,13 @@
     <t xml:space="preserve">So rechnen Sie die Folgeperiode ab (neuer Eigentümer ↔ Christine)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Blatt 'Zählerstände': Datum und Zählerstände zum neuen Stichtag in Spalte 'Stand 4' eintragen.</t>
+    <t xml:space="preserve">1. Blatt 'Zählerstände': Zählerstände zum 01.08.2026 in 'Stand 4' und zum Periodenende in 'Stand 5' eintragen.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Blatt 'Perioden', Zeile P3: Beginn, Ende, Monate und geleistete Zahlungen anpassen.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Blatt 'Abr_Folgeperiode': Ergebnis ablesen. Der Hauptwasseranschluss ist geteilt – über Christine laufen nur noch Heizung und Warmwasser; Kaltwasser ist daher aus. Die Schalter (1/0) lassen sich ändern.</t>
+    <t xml:space="preserve">3. Blatt 'Abr_Folgeperiode': Ergebnis ablesen. Ab August 2026 ist der Hauptwasseranschluss geteilt – über Christine laufen nur noch Heizung und Warmwasser; Kaltwasser ist daher aus. Die Schalter (1/0) lassen sich ändern.</t>
   </si>
   <si>
     <t xml:space="preserve">4. Blatt 'Eigentümer': Zahlung pro Monat eintragen, Saldo der Folgeperiode ablesen.</t>
@@ -193,7 +193,11 @@
   </si>
   <si>
     <t xml:space="preserve">Stichtag 4
-(Folgeperiode, noch offen)</t>
+(Start Folgeperiode, ca. 01.08.2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stichtag 5
+(Ende Folgeperiode, noch offen)</t>
   </si>
   <si>
     <t xml:space="preserve">Datum der Ablesung</t>
@@ -223,6 +227,9 @@
     <t xml:space="preserve">Stand 4</t>
   </si>
   <si>
+    <t xml:space="preserve">Stand 5</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hinweis</t>
   </si>
   <si>
@@ -304,7 +311,7 @@
     <t xml:space="preserve">Stand 2 nicht nötig (Kulanz rechnet Stand 1 bis 3)</t>
   </si>
   <si>
-    <t xml:space="preserve">Die Werte in Stand 1–3 stammen aus der Projekt-Zusammenfassung vom 19.06.2026 (vom Nutzer geliefert). Stand 4 ist für die Folgeperiode nach dem Eigentümerwechsel gedacht.</t>
+    <t xml:space="preserve">Die Werte in Stand 1–3 stammen aus der Projekt-Zusammenfassung vom 19.06.2026 (vom Nutzer geliefert). Stand 4 = Zählerstände zum 01.08.2026 (Beginn Folgeperiode), Stand 5 = Ende der Folgeperiode. Beltz bleibt bis 19.06.2026 unverändert.</t>
   </si>
   <si>
     <t xml:space="preserve">Kostensätze (Eingabe)</t>
@@ -502,7 +509,7 @@
     <t xml:space="preserve">P2 Ende 19.06.2026 = Stichtag der Abschlussabrechnung (~11 Monate).</t>
   </si>
   <si>
-    <t xml:space="preserve">P3 ist eine Platzhalter-Zeile für die Folgeperiode nach dem Eigentümerwechsel – Beginn, Ende, Monate und Zahlungen anpassen; Stichtag 4 in 'Zählerstände' eintragen.</t>
+    <t xml:space="preserve">P3 ist eine Platzhalter-Zeile für die Folgeperiode nach dem Eigentümerwechsel – Beginn, Ende, Monate und Zahlungen anpassen; Stand 4 (01.08.2026) und Stand 5 in 'Zählerstände' eintragen. Neue Berechnung ohne Kaltwasser gilt erst ab August 2026; davor (bis 19.06.2026 Beltz) unverändert.</t>
   </si>
   <si>
     <t xml:space="preserve">Maximal 24 Monate pro Periode (Monatsraster).</t>
@@ -1558,17 +1565,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="27" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B4" s="28" t="str">
         <f aca="false">Perioden!B9</f>
@@ -1577,16 +1584,16 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B5" s="24" t="n">
         <f aca="false">Perioden!C9</f>
-        <v>46193</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B6" s="24" t="n">
         <f aca="false">Perioden!D9</f>
@@ -1595,11 +1602,11 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B7" s="29" t="n">
         <f aca="false">Perioden!E9</f>
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1613,12 +1620,12 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>0</v>
@@ -1626,7 +1633,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>0</v>
@@ -1634,7 +1641,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>0</v>
@@ -1642,7 +1649,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>0</v>
@@ -1650,7 +1657,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C15" s="17" t="n">
         <v>0</v>
@@ -1658,7 +1665,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C16" s="17" t="n">
         <v>0</v>
@@ -1666,21 +1673,21 @@
     </row>
     <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="30" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B19" s="31" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C19" s="32" t="str">
         <f aca="false">IF(Berechnung!C9="","",ROUND(Berechnung!C9*Perioden!J9*Berechnung!I9*Kosten!B4,2))</f>
@@ -1689,10 +1696,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="30" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B20" s="31" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C20" s="32" t="str">
         <f aca="false">IF(Berechnung!H9="","",ROUND(Berechnung!H9*Kosten!B13,2))</f>
@@ -1701,10 +1708,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="30" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B21" s="31" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C21" s="32" t="str">
         <f aca="false">IF(Berechnung!H9="","",ROUND(Berechnung!H9/Perioden!E9*SUMIFS(Monatsraster!$E$5:$E$100,Monatsraster!$A$5:$A$100,Perioden!$A$9),2))</f>
@@ -1713,10 +1720,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="30" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B22" s="31" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C22" s="32" t="n">
         <f aca="false">IF(C11=0,0,IF(Berechnung!G9="","",ROUND(Berechnung!G9/Perioden!E9*SUMIFS(Monatsraster!$E$5:$E$100,Monatsraster!$A$5:$A$100,Perioden!$A$9),2)))</f>
@@ -1725,10 +1732,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="30" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B23" s="31" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C23" s="32" t="n">
         <f aca="false">IF(C12=0,0,IF(Berechnung!D9="","",ROUND(Berechnung!D9*Perioden!J9*Kosten!B4,2)))</f>
@@ -1737,10 +1744,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="30" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B24" s="31" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C24" s="32" t="n">
         <f aca="false">IF(C13=0,0,ROUND(Perioden!K9*Kosten!B7,2))</f>
@@ -1749,10 +1756,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="30" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B25" s="31" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C25" s="32" t="n">
         <f aca="false">IF(C14=0,0,ROUND(Kosten!B14*Perioden!E9,2))</f>
@@ -1761,10 +1768,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="30" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B26" s="31" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C26" s="32" t="n">
         <f aca="false">IF(C15=0,0,ROUND(Kosten!B16*Perioden!E9,2))</f>
@@ -1773,10 +1780,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="30" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B27" s="31" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C27" s="32" t="n">
         <f aca="false">IF(C16=0,0,ROUND(SUMIFS(Monatsraster!$F$5:$F$100,Monatsraster!$A$5:$A$100,Perioden!$A$9),2))</f>
@@ -1785,7 +1792,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="33" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B28" s="34"/>
       <c r="C28" s="35" t="str">
@@ -1795,7 +1802,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C29" s="9" t="n">
         <f aca="false">Perioden!G9</f>
@@ -1809,13 +1816,13 @@
       </c>
       <c r="B30" s="34"/>
       <c r="C30" s="35" t="str">
-        <f aca="false">IF(C28="","Stand 4 fehlt",C28-C29)</f>
-        <v>Stand 4 fehlt</v>
+        <f aca="false">IF(C28="","Stand 5 fehlt",C28-C29)</f>
+        <v>Stand 5 fehlt</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -1843,33 +1850,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>195</v>
@@ -1877,7 +1884,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>195</v>
@@ -1885,12 +1892,12 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>500</v>
@@ -1898,7 +1905,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>273</v>
@@ -1906,7 +1913,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>210.74</v>
@@ -1914,7 +1921,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>104</v>
@@ -1922,7 +1929,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B15" s="36" t="n">
         <f aca="false">SUM(B11:B14)</f>
@@ -1931,7 +1938,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>81.99</v>
@@ -1939,15 +1946,15 @@
     </row>
     <row r="19" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B20" s="9" t="n">
         <f aca="false">ROUND(Abr_P1_Felix!C22-Perioden!E6*B7,2)</f>
@@ -1956,7 +1963,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B21" s="9" t="n">
         <f aca="false">Abr_Leerstand!C17</f>
@@ -1965,7 +1972,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B22" s="9" t="n">
         <f aca="false">ROUND(Abr_P2_Beltz!C21-Perioden!E8*B8,2)</f>
@@ -1974,7 +1981,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B23" s="36" t="n">
         <f aca="false">SUM(B20:B22)</f>
@@ -1983,7 +1990,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B24" s="9" t="n">
         <f aca="false">B15</f>
@@ -1992,7 +1999,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B25" s="9" t="n">
         <f aca="false">B16</f>
@@ -2001,7 +2008,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="33" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B26" s="35" t="n">
         <f aca="false">B23+B24+B25</f>
@@ -2010,12 +2017,12 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B29" s="26" t="n">
         <f aca="false">Zählerstände!G12-Zählerstände!E12</f>
@@ -2024,7 +2031,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B30" s="9" t="n">
         <f aca="false">ROUND(B29*Kosten!B13,2)</f>
@@ -2038,7 +2045,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B33" s="8" t="n">
         <v>0</v>
@@ -2046,7 +2053,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B34" s="7" t="str">
         <f aca="false">Abr_Folgeperiode!C28</f>
@@ -2055,7 +2062,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B35" s="36" t="str">
         <f aca="false">IF(B34="","",B34-Perioden!E9*B33)</f>
@@ -2064,27 +2071,27 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -2115,32 +2122,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3953,7 +3960,7 @@
       </c>
       <c r="C77" s="38" t="n">
         <f aca="false">IF(B77&lt;=Perioden!$E$9,EDATE(Perioden!$C$9,B77-1),"")</f>
-        <v>46193</v>
+        <v>46235</v>
       </c>
       <c r="D77" s="37" t="n">
         <f aca="false">IF(C77="","",YEAR(C77))</f>
@@ -3978,7 +3985,7 @@
       </c>
       <c r="C78" s="38" t="n">
         <f aca="false">IF(B78&lt;=Perioden!$E$9,EDATE(Perioden!$C$9,B78-1),"")</f>
-        <v>46223</v>
+        <v>46266</v>
       </c>
       <c r="D78" s="37" t="n">
         <f aca="false">IF(C78="","",YEAR(C78))</f>
@@ -4003,7 +4010,7 @@
       </c>
       <c r="C79" s="38" t="n">
         <f aca="false">IF(B79&lt;=Perioden!$E$9,EDATE(Perioden!$C$9,B79-1),"")</f>
-        <v>46254</v>
+        <v>46296</v>
       </c>
       <c r="D79" s="37" t="n">
         <f aca="false">IF(C79="","",YEAR(C79))</f>
@@ -4028,7 +4035,7 @@
       </c>
       <c r="C80" s="38" t="n">
         <f aca="false">IF(B80&lt;=Perioden!$E$9,EDATE(Perioden!$C$9,B80-1),"")</f>
-        <v>46285</v>
+        <v>46327</v>
       </c>
       <c r="D80" s="37" t="n">
         <f aca="false">IF(C80="","",YEAR(C80))</f>
@@ -4053,7 +4060,7 @@
       </c>
       <c r="C81" s="38" t="n">
         <f aca="false">IF(B81&lt;=Perioden!$E$9,EDATE(Perioden!$C$9,B81-1),"")</f>
-        <v>46315</v>
+        <v>46357</v>
       </c>
       <c r="D81" s="37" t="n">
         <f aca="false">IF(C81="","",YEAR(C81))</f>
@@ -4076,21 +4083,21 @@
       <c r="B82" s="37" t="n">
         <v>6</v>
       </c>
-      <c r="C82" s="38" t="n">
+      <c r="C82" s="38" t="str">
         <f aca="false">IF(B82&lt;=Perioden!$E$9,EDATE(Perioden!$C$9,B82-1),"")</f>
-        <v>46346</v>
-      </c>
-      <c r="D82" s="37" t="n">
+        <v/>
+      </c>
+      <c r="D82" s="37" t="str">
         <f aca="false">IF(C82="","",YEAR(C82))</f>
-        <v>2026</v>
+        <v/>
       </c>
       <c r="E82" s="22" t="n">
         <f aca="false">IF(C82="",0,INDEX(Kosten!$B$21:$B$27,MATCH(D82,Kosten!$A$21:$A$27,0)))</f>
-        <v>7.44</v>
+        <v>0</v>
       </c>
       <c r="F82" s="22" t="n">
         <f aca="false">IF(C82="",0,INDEX(Kosten!$D$21:$D$27,MATCH(D82,Kosten!$A$21:$A$27,0)))</f>
-        <v>4.97</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4721,7 +4728,7 @@
       </c>
       <c r="D9" s="7" t="str">
         <f aca="false">Abr_Folgeperiode!C30</f>
-        <v>Stand 4 fehlt</v>
+        <v>Stand 5 fehlt</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>39</v>
@@ -4801,7 +4808,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -4811,8 +4818,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4838,10 +4845,13 @@
       <c r="H3" s="5" t="s">
         <v>52</v>
       </c>
+      <c r="I3" s="5" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>45323</v>
@@ -4852,49 +4862,55 @@
       <c r="G4" s="14" t="n">
         <v>46192</v>
       </c>
-      <c r="H4" s="14"/>
+      <c r="H4" s="14" t="n">
+        <v>46235</v>
+      </c>
+      <c r="I4" s="14"/>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E6" s="15" t="n">
         <v>17705.44</v>
@@ -4906,20 +4922,21 @@
         <v>40467.3</v>
       </c>
       <c r="H6" s="15"/>
-      <c r="I6" s="4"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>68</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="E7" s="15" t="n">
         <v>3396.16</v>
@@ -4931,20 +4948,21 @@
         <v>7599.68</v>
       </c>
       <c r="H7" s="15"/>
-      <c r="I7" s="4"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E8" s="15" t="n">
         <v>32.5</v>
@@ -4956,22 +4974,23 @@
         <v>66.322</v>
       </c>
       <c r="H8" s="15"/>
-      <c r="I8" s="4" t="s">
-        <v>74</v>
+      <c r="I8" s="15"/>
+      <c r="J8" s="4" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>75</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>73</v>
       </c>
       <c r="E9" s="15" t="n">
         <v>33</v>
@@ -4983,20 +5002,21 @@
         <v>60.394</v>
       </c>
       <c r="H9" s="15"/>
-      <c r="I9" s="4"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E10" s="15" t="n">
         <v>61.904</v>
@@ -5008,20 +5028,21 @@
         <v>149.138</v>
       </c>
       <c r="H10" s="15"/>
-      <c r="I10" s="4"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B11" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>81</v>
       </c>
       <c r="E11" s="15" t="n">
         <v>35.021</v>
@@ -5033,20 +5054,21 @@
         <v>63.495</v>
       </c>
       <c r="H11" s="15"/>
-      <c r="I11" s="4"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E12" s="15" t="n">
         <v>6.569</v>
@@ -5056,13 +5078,14 @@
         <v>120.116</v>
       </c>
       <c r="H12" s="15"/>
-      <c r="I12" s="4" t="s">
-        <v>88</v>
+      <c r="I12" s="15"/>
+      <c r="J12" s="4" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -5093,66 +5116,66 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B4" s="16" t="n">
         <v>0.2462</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B5" s="17" t="n">
         <v>88</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B6" s="17" t="n">
         <v>270</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B7" s="18" t="n">
         <f aca="false">B5/B6</f>
@@ -5160,170 +5183,170 @@
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>563.11</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>375.41</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B10" s="17" t="n">
         <v>8</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">B9/B10</f>
         <v>46.92625</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B12" s="19" t="n">
         <v>20.9</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B13" s="20" t="n">
         <f aca="false">B12*B4</f>
         <v>5.14558</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>24.18</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D14" s="4"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>188.78</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">B15/12</f>
         <v>15.7316666666667</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D16" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B17" s="17" t="n">
         <v>226</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>80</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5373,7 +5396,7 @@
         <v>4.97</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5391,7 +5414,7 @@
         <v>4.97</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5409,7 +5432,7 @@
         <v>4.97</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5427,7 +5450,7 @@
         <v>4.97</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5445,12 +5468,12 @@
         <v>4.97</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -5485,61 +5508,61 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C6" s="14" t="n">
         <v>45323</v>
@@ -5570,17 +5593,17 @@
         <v>563.11</v>
       </c>
       <c r="L6" s="24" t="n">
-        <f aca="false">INDEX(Zählerstände!$E$4:$H$4,H6)</f>
+        <f aca="false">INDEX(Zählerstände!$E$4:$I$4,H6)</f>
         <v>45323</v>
       </c>
       <c r="M6" s="24" t="n">
-        <f aca="false">INDEX(Zählerstände!$E$4:$H$4,I6)</f>
+        <f aca="false">INDEX(Zählerstände!$E$4:$I$4,I6)</f>
         <v>45778</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B7" s="23" t="s">
         <v>35</v>
@@ -5615,20 +5638,20 @@
         <v>140.77875</v>
       </c>
       <c r="L7" s="24" t="n">
-        <f aca="false">INDEX(Zählerstände!$E$4:$H$4,H7)</f>
+        <f aca="false">INDEX(Zählerstände!$E$4:$I$4,H7)</f>
         <v>45778</v>
       </c>
       <c r="M7" s="24" t="n">
-        <f aca="false">INDEX(Zählerstände!$E$4:$H$4,I7)</f>
+        <f aca="false">INDEX(Zählerstände!$E$4:$I$4,I7)</f>
         <v>46192</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>45870</v>
@@ -5661,29 +5684,29 @@
         <v>516.18875</v>
       </c>
       <c r="L8" s="24" t="n">
-        <f aca="false">INDEX(Zählerstände!$E$4:$H$4,H8)</f>
+        <f aca="false">INDEX(Zählerstände!$E$4:$I$4,H8)</f>
         <v>45778</v>
       </c>
       <c r="M8" s="24" t="n">
-        <f aca="false">INDEX(Zählerstände!$E$4:$H$4,I8)</f>
+        <f aca="false">INDEX(Zählerstände!$E$4:$I$4,I8)</f>
         <v>46192</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C9" s="14" t="n">
-        <v>46193</v>
+        <v>46235</v>
       </c>
       <c r="D9" s="14" t="n">
         <v>46387</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>0</v>
@@ -5692,50 +5715,50 @@
         <v>0</v>
       </c>
       <c r="H9" s="17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I9" s="17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J9" s="16" t="n">
         <v>1</v>
       </c>
       <c r="K9" s="9" t="n">
         <f aca="false">Kosten!B11*E9</f>
-        <v>281.5575</v>
+        <v>234.63125</v>
       </c>
       <c r="L9" s="24" t="n">
-        <f aca="false">INDEX(Zählerstände!$E$4:$H$4,H9)</f>
-        <v>46192</v>
+        <f aca="false">INDEX(Zählerstände!$E$4:$I$4,H9)</f>
+        <v>46235</v>
       </c>
       <c r="M9" s="24" t="n">
-        <f aca="false">INDEX(Zählerstände!$E$4:$H$4,I9)</f>
+        <f aca="false">INDEX(Zählerstände!$E$4:$I$4,I9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -5770,38 +5793,38 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>27</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>43</v>
@@ -5810,7 +5833,7 @@
         <v>44</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5823,27 +5846,27 @@
         <v>Felix Adameck</v>
       </c>
       <c r="C6" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$6:$H$6,Perioden!$H6),INDEX(Zählerstände!$E$6:$H$6,Perioden!$I6))&lt;2,"",INDEX(Zählerstände!$E$6:$H$6,Perioden!$I6)-INDEX(Zählerstände!$E$6:$H$6,Perioden!$H6))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$6:$I$6,Perioden!$H6),INDEX(Zählerstände!$E$6:$I$6,Perioden!$I6))&lt;2,"",INDEX(Zählerstände!$E$6:$I$6,Perioden!$I6)-INDEX(Zählerstände!$E$6:$I$6,Perioden!$H6))</f>
         <v>11356.82</v>
       </c>
       <c r="D6" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$7:$H$7,Perioden!$H6),INDEX(Zählerstände!$E$7:$H$7,Perioden!$I6))&lt;2,"",INDEX(Zählerstände!$E$7:$H$7,Perioden!$I6)-INDEX(Zählerstände!$E$7:$H$7,Perioden!$H6))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$7:$I$7,Perioden!$H6),INDEX(Zählerstände!$E$7:$I$7,Perioden!$I6))&lt;2,"",INDEX(Zählerstände!$E$7:$I$7,Perioden!$I6)-INDEX(Zählerstände!$E$7:$I$7,Perioden!$H6))</f>
         <v>2084.74</v>
       </c>
       <c r="E6" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$8:$H$8,Perioden!$H6),INDEX(Zählerstände!$E$8:$H$8,Perioden!$I6))&lt;2,"",INDEX(Zählerstände!$E$8:$H$8,Perioden!$I6)-INDEX(Zählerstände!$E$8:$H$8,Perioden!$H6))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$8:$I$8,Perioden!$H6),INDEX(Zählerstände!$E$8:$I$8,Perioden!$I6))&lt;2,"",INDEX(Zählerstände!$E$8:$I$8,Perioden!$I6)-INDEX(Zählerstände!$E$8:$I$8,Perioden!$H6))</f>
         <v>17.45</v>
       </c>
       <c r="F6" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$9:$H$9,Perioden!$H6),INDEX(Zählerstände!$E$9:$H$9,Perioden!$I6))&lt;2,"",INDEX(Zählerstände!$E$9:$H$9,Perioden!$I6)-INDEX(Zählerstände!$E$9:$H$9,Perioden!$H6))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$9:$I$9,Perioden!$H6),INDEX(Zählerstände!$E$9:$I$9,Perioden!$I6))&lt;2,"",INDEX(Zählerstände!$E$9:$I$9,Perioden!$I6)-INDEX(Zählerstände!$E$9:$I$9,Perioden!$H6))</f>
         <v>20</v>
       </c>
       <c r="G6" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$10:$H$10,Perioden!$H6),INDEX(Zählerstände!$E$10:$H$10,Perioden!$I6))&lt;2,"",INDEX(Zählerstände!$E$10:$H$10,Perioden!$I6)-INDEX(Zählerstände!$E$10:$H$10,Perioden!$H6))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$10:$I$10,Perioden!$H6),INDEX(Zählerstände!$E$10:$I$10,Perioden!$I6))&lt;2,"",INDEX(Zählerstände!$E$10:$I$10,Perioden!$I6)-INDEX(Zählerstände!$E$10:$I$10,Perioden!$H6))</f>
         <v>45.906</v>
       </c>
       <c r="H6" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$11:$H$11,Perioden!$H6),INDEX(Zählerstände!$E$11:$H$11,Perioden!$I6))&lt;2,"",INDEX(Zählerstände!$E$11:$H$11,Perioden!$I6)-INDEX(Zählerstände!$E$11:$H$11,Perioden!$H6))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$11:$I$11,Perioden!$H6),INDEX(Zählerstände!$E$11:$I$11,Perioden!$I6))&lt;2,"",INDEX(Zählerstände!$E$11:$I$11,Perioden!$I6)-INDEX(Zählerstände!$E$11:$I$11,Perioden!$H6))</f>
         <v>18.049</v>
       </c>
       <c r="I6" s="18" t="n">
@@ -5869,27 +5892,27 @@
         <v>Leerstand (Thomas Weis)</v>
       </c>
       <c r="C7" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$6:$H$6,Perioden!$H7),INDEX(Zählerstände!$E$6:$H$6,Perioden!$I7))&lt;2,"",INDEX(Zählerstände!$E$6:$H$6,Perioden!$I7)-INDEX(Zählerstände!$E$6:$H$6,Perioden!$H7))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$6:$I$6,Perioden!$H7),INDEX(Zählerstände!$E$6:$I$6,Perioden!$I7))&lt;2,"",INDEX(Zählerstände!$E$6:$I$6,Perioden!$I7)-INDEX(Zählerstände!$E$6:$I$6,Perioden!$H7))</f>
         <v>11405.04</v>
       </c>
       <c r="D7" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$7:$H$7,Perioden!$H7),INDEX(Zählerstände!$E$7:$H$7,Perioden!$I7))&lt;2,"",INDEX(Zählerstände!$E$7:$H$7,Perioden!$I7)-INDEX(Zählerstände!$E$7:$H$7,Perioden!$H7))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$7:$I$7,Perioden!$H7),INDEX(Zählerstände!$E$7:$I$7,Perioden!$I7))&lt;2,"",INDEX(Zählerstände!$E$7:$I$7,Perioden!$I7)-INDEX(Zählerstände!$E$7:$I$7,Perioden!$H7))</f>
         <v>2118.78</v>
       </c>
       <c r="E7" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$8:$H$8,Perioden!$H7),INDEX(Zählerstände!$E$8:$H$8,Perioden!$I7))&lt;2,"",INDEX(Zählerstände!$E$8:$H$8,Perioden!$I7)-INDEX(Zählerstände!$E$8:$H$8,Perioden!$H7))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$8:$I$8,Perioden!$H7),INDEX(Zählerstände!$E$8:$I$8,Perioden!$I7))&lt;2,"",INDEX(Zählerstände!$E$8:$I$8,Perioden!$I7)-INDEX(Zählerstände!$E$8:$I$8,Perioden!$H7))</f>
         <v>16.372</v>
       </c>
       <c r="F7" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$9:$H$9,Perioden!$H7),INDEX(Zählerstände!$E$9:$H$9,Perioden!$I7))&lt;2,"",INDEX(Zählerstände!$E$9:$H$9,Perioden!$I7)-INDEX(Zählerstände!$E$9:$H$9,Perioden!$H7))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$9:$I$9,Perioden!$H7),INDEX(Zählerstände!$E$9:$I$9,Perioden!$I7))&lt;2,"",INDEX(Zählerstände!$E$9:$I$9,Perioden!$I7)-INDEX(Zählerstände!$E$9:$I$9,Perioden!$H7))</f>
         <v>7.394</v>
       </c>
       <c r="G7" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$10:$H$10,Perioden!$H7),INDEX(Zählerstände!$E$10:$H$10,Perioden!$I7))&lt;2,"",INDEX(Zählerstände!$E$10:$H$10,Perioden!$I7)-INDEX(Zählerstände!$E$10:$H$10,Perioden!$H7))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$10:$I$10,Perioden!$H7),INDEX(Zählerstände!$E$10:$I$10,Perioden!$I7))&lt;2,"",INDEX(Zählerstände!$E$10:$I$10,Perioden!$I7)-INDEX(Zählerstände!$E$10:$I$10,Perioden!$H7))</f>
         <v>41.328</v>
       </c>
       <c r="H7" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$11:$H$11,Perioden!$H7),INDEX(Zählerstände!$E$11:$H$11,Perioden!$I7))&lt;2,"",INDEX(Zählerstände!$E$11:$H$11,Perioden!$I7)-INDEX(Zählerstände!$E$11:$H$11,Perioden!$H7))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$11:$I$11,Perioden!$H7),INDEX(Zählerstände!$E$11:$I$11,Perioden!$I7))&lt;2,"",INDEX(Zählerstände!$E$11:$I$11,Perioden!$I7)-INDEX(Zählerstände!$E$11:$I$11,Perioden!$H7))</f>
         <v>10.425</v>
       </c>
       <c r="I7" s="18" t="n">
@@ -5915,27 +5938,27 @@
         <v>Fam. Kristin &amp; Maximilian Beltz</v>
       </c>
       <c r="C8" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$6:$H$6,Perioden!$H8),INDEX(Zählerstände!$E$6:$H$6,Perioden!$I8))&lt;2,"",INDEX(Zählerstände!$E$6:$H$6,Perioden!$I8)-INDEX(Zählerstände!$E$6:$H$6,Perioden!$H8))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$6:$I$6,Perioden!$H8),INDEX(Zählerstände!$E$6:$I$6,Perioden!$I8))&lt;2,"",INDEX(Zählerstände!$E$6:$I$6,Perioden!$I8)-INDEX(Zählerstände!$E$6:$I$6,Perioden!$H8))</f>
         <v>11405.04</v>
       </c>
       <c r="D8" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$7:$H$7,Perioden!$H8),INDEX(Zählerstände!$E$7:$H$7,Perioden!$I8))&lt;2,"",INDEX(Zählerstände!$E$7:$H$7,Perioden!$I8)-INDEX(Zählerstände!$E$7:$H$7,Perioden!$H8))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$7:$I$7,Perioden!$H8),INDEX(Zählerstände!$E$7:$I$7,Perioden!$I8))&lt;2,"",INDEX(Zählerstände!$E$7:$I$7,Perioden!$I8)-INDEX(Zählerstände!$E$7:$I$7,Perioden!$H8))</f>
         <v>2118.78</v>
       </c>
       <c r="E8" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$8:$H$8,Perioden!$H8),INDEX(Zählerstände!$E$8:$H$8,Perioden!$I8))&lt;2,"",INDEX(Zählerstände!$E$8:$H$8,Perioden!$I8)-INDEX(Zählerstände!$E$8:$H$8,Perioden!$H8))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$8:$I$8,Perioden!$H8),INDEX(Zählerstände!$E$8:$I$8,Perioden!$I8))&lt;2,"",INDEX(Zählerstände!$E$8:$I$8,Perioden!$I8)-INDEX(Zählerstände!$E$8:$I$8,Perioden!$H8))</f>
         <v>16.372</v>
       </c>
       <c r="F8" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$9:$H$9,Perioden!$H8),INDEX(Zählerstände!$E$9:$H$9,Perioden!$I8))&lt;2,"",INDEX(Zählerstände!$E$9:$H$9,Perioden!$I8)-INDEX(Zählerstände!$E$9:$H$9,Perioden!$H8))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$9:$I$9,Perioden!$H8),INDEX(Zählerstände!$E$9:$I$9,Perioden!$I8))&lt;2,"",INDEX(Zählerstände!$E$9:$I$9,Perioden!$I8)-INDEX(Zählerstände!$E$9:$I$9,Perioden!$H8))</f>
         <v>7.394</v>
       </c>
       <c r="G8" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$10:$H$10,Perioden!$H8),INDEX(Zählerstände!$E$10:$H$10,Perioden!$I8))&lt;2,"",INDEX(Zählerstände!$E$10:$H$10,Perioden!$I8)-INDEX(Zählerstände!$E$10:$H$10,Perioden!$H8))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$10:$I$10,Perioden!$H8),INDEX(Zählerstände!$E$10:$I$10,Perioden!$I8))&lt;2,"",INDEX(Zählerstände!$E$10:$I$10,Perioden!$I8)-INDEX(Zählerstände!$E$10:$I$10,Perioden!$H8))</f>
         <v>41.328</v>
       </c>
       <c r="H8" s="26" t="n">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$11:$H$11,Perioden!$H8),INDEX(Zählerstände!$E$11:$H$11,Perioden!$I8))&lt;2,"",INDEX(Zählerstände!$E$11:$H$11,Perioden!$I8)-INDEX(Zählerstände!$E$11:$H$11,Perioden!$H8))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$11:$I$11,Perioden!$H8),INDEX(Zählerstände!$E$11:$I$11,Perioden!$I8))&lt;2,"",INDEX(Zählerstände!$E$11:$I$11,Perioden!$I8)-INDEX(Zählerstände!$E$11:$I$11,Perioden!$H8))</f>
         <v>10.425</v>
       </c>
       <c r="I8" s="18" t="n">
@@ -5961,27 +5984,27 @@
         <v>Neuer Eigentümer (Name folgt) – Folgeperiode</v>
       </c>
       <c r="C9" s="26" t="str">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$6:$H$6,Perioden!$H9),INDEX(Zählerstände!$E$6:$H$6,Perioden!$I9))&lt;2,"",INDEX(Zählerstände!$E$6:$H$6,Perioden!$I9)-INDEX(Zählerstände!$E$6:$H$6,Perioden!$H9))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$6:$I$6,Perioden!$H9),INDEX(Zählerstände!$E$6:$I$6,Perioden!$I9))&lt;2,"",INDEX(Zählerstände!$E$6:$I$6,Perioden!$I9)-INDEX(Zählerstände!$E$6:$I$6,Perioden!$H9))</f>
         <v/>
       </c>
       <c r="D9" s="26" t="str">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$7:$H$7,Perioden!$H9),INDEX(Zählerstände!$E$7:$H$7,Perioden!$I9))&lt;2,"",INDEX(Zählerstände!$E$7:$H$7,Perioden!$I9)-INDEX(Zählerstände!$E$7:$H$7,Perioden!$H9))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$7:$I$7,Perioden!$H9),INDEX(Zählerstände!$E$7:$I$7,Perioden!$I9))&lt;2,"",INDEX(Zählerstände!$E$7:$I$7,Perioden!$I9)-INDEX(Zählerstände!$E$7:$I$7,Perioden!$H9))</f>
         <v/>
       </c>
       <c r="E9" s="26" t="str">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$8:$H$8,Perioden!$H9),INDEX(Zählerstände!$E$8:$H$8,Perioden!$I9))&lt;2,"",INDEX(Zählerstände!$E$8:$H$8,Perioden!$I9)-INDEX(Zählerstände!$E$8:$H$8,Perioden!$H9))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$8:$I$8,Perioden!$H9),INDEX(Zählerstände!$E$8:$I$8,Perioden!$I9))&lt;2,"",INDEX(Zählerstände!$E$8:$I$8,Perioden!$I9)-INDEX(Zählerstände!$E$8:$I$8,Perioden!$H9))</f>
         <v/>
       </c>
       <c r="F9" s="26" t="str">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$9:$H$9,Perioden!$H9),INDEX(Zählerstände!$E$9:$H$9,Perioden!$I9))&lt;2,"",INDEX(Zählerstände!$E$9:$H$9,Perioden!$I9)-INDEX(Zählerstände!$E$9:$H$9,Perioden!$H9))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$9:$I$9,Perioden!$H9),INDEX(Zählerstände!$E$9:$I$9,Perioden!$I9))&lt;2,"",INDEX(Zählerstände!$E$9:$I$9,Perioden!$I9)-INDEX(Zählerstände!$E$9:$I$9,Perioden!$H9))</f>
         <v/>
       </c>
       <c r="G9" s="26" t="str">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$10:$H$10,Perioden!$H9),INDEX(Zählerstände!$E$10:$H$10,Perioden!$I9))&lt;2,"",INDEX(Zählerstände!$E$10:$H$10,Perioden!$I9)-INDEX(Zählerstände!$E$10:$H$10,Perioden!$H9))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$10:$I$10,Perioden!$H9),INDEX(Zählerstände!$E$10:$I$10,Perioden!$I9))&lt;2,"",INDEX(Zählerstände!$E$10:$I$10,Perioden!$I9)-INDEX(Zählerstände!$E$10:$I$10,Perioden!$H9))</f>
         <v/>
       </c>
       <c r="H9" s="26" t="str">
-        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$11:$H$11,Perioden!$H9),INDEX(Zählerstände!$E$11:$H$11,Perioden!$I9))&lt;2,"",INDEX(Zählerstände!$E$11:$H$11,Perioden!$I9)-INDEX(Zählerstände!$E$11:$H$11,Perioden!$H9))</f>
+        <f aca="false">IF(COUNT(INDEX(Zählerstände!$E$11:$I$11,Perioden!$H9),INDEX(Zählerstände!$E$11:$I$11,Perioden!$I9))&lt;2,"",INDEX(Zählerstände!$E$11:$I$11,Perioden!$I9)-INDEX(Zählerstände!$E$11:$I$11,Perioden!$H9))</f>
         <v/>
       </c>
       <c r="I9" s="18" t="str">
@@ -5999,7 +6022,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -6028,17 +6051,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="27" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B4" s="28" t="str">
         <f aca="false">Perioden!B6</f>
@@ -6047,7 +6070,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B5" s="24" t="n">
         <f aca="false">Perioden!C6</f>
@@ -6056,7 +6079,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B6" s="24" t="n">
         <f aca="false">Perioden!D6</f>
@@ -6065,7 +6088,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B7" s="29" t="n">
         <f aca="false">Perioden!E6</f>
@@ -6083,21 +6106,21 @@
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="30" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C11" s="32" t="n">
         <f aca="false">ROUND(Berechnung!C6*Perioden!J6*Berechnung!I6*Kosten!B4,2)</f>
@@ -6106,10 +6129,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="30" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B12" s="31" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C12" s="32" t="n">
         <f aca="false">ROUND(Berechnung!H6*Kosten!B13,2)</f>
@@ -6118,10 +6141,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="30" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B13" s="31" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C13" s="32" t="n">
         <f aca="false">ROUND(Berechnung!D6*Perioden!J6*Kosten!B4,2)</f>
@@ -6130,10 +6153,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="30" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B14" s="31" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C14" s="32" t="n">
         <f aca="false">ROUND(Perioden!K6*Kosten!B7,2)</f>
@@ -6146,7 +6169,7 @@
         <v>Wasser/Abwasser 2024</v>
       </c>
       <c r="B15" s="31" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C15" s="32" t="n">
         <f aca="false">ROUND((Berechnung!G6+Berechnung!H6)/Perioden!E6*SUMIFS(Monatsraster!$E$5:$E$100,Monatsraster!$A$5:$A$100,Perioden!$A$6,Monatsraster!$D$5:$D$100,YEAR(Perioden!$C$6)),2)</f>
@@ -6159,7 +6182,7 @@
         <v>Wasser/Abwasser 2025</v>
       </c>
       <c r="B16" s="31" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C16" s="32" t="n">
         <f aca="false">ROUND((Berechnung!G6+Berechnung!H6)/Perioden!E6*SUMIFS(Monatsraster!$E$5:$E$100,Monatsraster!$A$5:$A$100,Perioden!$A$6,Monatsraster!$D$5:$D$100,YEAR(Perioden!$C$6)+1),2)</f>
@@ -6168,10 +6191,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="30" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B17" s="31" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C17" s="32" t="n">
         <f aca="false">ROUND(Kosten!B14*Perioden!E6,2)</f>
@@ -6180,10 +6203,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="30" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B18" s="31" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C18" s="32" t="n">
         <f aca="false">ROUND(Kosten!B16*Perioden!E6,2)</f>
@@ -6196,7 +6219,7 @@
         <v>Niederschlagswasser 2024</v>
       </c>
       <c r="B19" s="31" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C19" s="32" t="n">
         <f aca="false">ROUND(SUMIFS(Monatsraster!$F$5:$F$100,Monatsraster!$A$5:$A$100,Perioden!$A$6,Monatsraster!$D$5:$D$100,YEAR(Perioden!$C$6)),2)</f>
@@ -6209,7 +6232,7 @@
         <v>Niederschlagswasser 2025</v>
       </c>
       <c r="B20" s="31" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C20" s="32" t="n">
         <f aca="false">ROUND(SUMIFS(Monatsraster!$F$5:$F$100,Monatsraster!$A$5:$A$100,Perioden!$A$6,Monatsraster!$D$5:$D$100,YEAR(Perioden!$C$6)+1),2)</f>
@@ -6218,7 +6241,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="33" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B21" s="34"/>
       <c r="C21" s="35" t="n">
@@ -6228,7 +6251,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="33" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B22" s="34"/>
       <c r="C22" s="35" t="n">
@@ -6238,7 +6261,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C23" s="9" t="n">
         <f aca="false">Perioden!G6</f>
@@ -6258,7 +6281,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -6287,17 +6310,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="27" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B4" s="28" t="str">
         <f aca="false">Perioden!B7</f>
@@ -6306,7 +6329,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B5" s="24" t="n">
         <f aca="false">Perioden!C7</f>
@@ -6315,7 +6338,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B6" s="24" t="n">
         <f aca="false">Perioden!D7</f>
@@ -6324,7 +6347,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B7" s="29" t="n">
         <f aca="false">Perioden!E7</f>
@@ -6342,21 +6365,21 @@
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="30" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C11" s="32" t="n">
         <f aca="false">ROUND(Berechnung!C7*Perioden!J7*Berechnung!I7*Kosten!B4,2)</f>
@@ -6365,10 +6388,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="30" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B12" s="31" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C12" s="32" t="n">
         <f aca="false">ROUND(Berechnung!D7*Perioden!J7*Kosten!B4,2)</f>
@@ -6377,10 +6400,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="30" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B13" s="31" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C13" s="32" t="n">
         <f aca="false">ROUND(Perioden!K7*Kosten!B7,2)</f>
@@ -6389,10 +6412,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="30" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B14" s="31" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C14" s="32" t="n">
         <f aca="false">ROUND(Kosten!B14*Perioden!E7,2)</f>
@@ -6401,10 +6424,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="30" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B15" s="31" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C15" s="32" t="n">
         <f aca="false">ROUND(Kosten!B16*Perioden!E7,2)</f>
@@ -6413,10 +6436,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="30" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B16" s="31" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C16" s="32" t="n">
         <f aca="false">ROUND(SUMIFS(Monatsraster!$F$5:$F$100,Monatsraster!$A$5:$A$100,Perioden!$A$7),2)</f>
@@ -6425,7 +6448,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="33" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B17" s="34"/>
       <c r="C17" s="35" t="n">
@@ -6459,17 +6482,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="27" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B4" s="28" t="str">
         <f aca="false">Perioden!B8</f>
@@ -6478,7 +6501,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B5" s="24" t="n">
         <f aca="false">Perioden!C8</f>
@@ -6487,7 +6510,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B6" s="24" t="n">
         <f aca="false">Perioden!D8</f>
@@ -6496,7 +6519,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B7" s="29" t="n">
         <f aca="false">Perioden!E8</f>
@@ -6514,21 +6537,21 @@
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="30" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C11" s="32" t="n">
         <f aca="false">ROUND(Berechnung!C8*Perioden!J8*Berechnung!I8*Kosten!B4,2)</f>
@@ -6537,10 +6560,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="30" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B12" s="31" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C12" s="32" t="n">
         <f aca="false">ROUND(Berechnung!H8*Kosten!B13,2)</f>
@@ -6549,10 +6572,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="30" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B13" s="31" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C13" s="32" t="n">
         <f aca="false">ROUND(Berechnung!D8*Perioden!J8*Kosten!B4,2)</f>
@@ -6561,10 +6584,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="30" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B14" s="31" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C14" s="32" t="n">
         <f aca="false">ROUND(Perioden!K8*Kosten!B7,2)</f>
@@ -6573,10 +6596,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="30" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B15" s="31" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C15" s="32" t="n">
         <f aca="false">ROUND((Berechnung!G8+Berechnung!H8)/Perioden!E8*SUMIFS(Monatsraster!$E$5:$E$100,Monatsraster!$A$5:$A$100,Perioden!$A$8),2)</f>
@@ -6585,10 +6608,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="30" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B16" s="31" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C16" s="32" t="n">
         <f aca="false">ROUND(Kosten!B14*Perioden!E8,2)</f>
@@ -6597,10 +6620,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="30" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B17" s="31" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C17" s="32" t="n">
         <f aca="false">ROUND(Kosten!B16*Perioden!E8,2)</f>
@@ -6609,10 +6632,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="30" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B18" s="31" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C18" s="32" t="n">
         <f aca="false">ROUND(SUMIFS(Monatsraster!$F$5:$F$100,Monatsraster!$A$5:$A$100,Perioden!$A$8),2)</f>
@@ -6621,7 +6644,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="33" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B19" s="34"/>
       <c r="C19" s="35" t="n">
@@ -6631,7 +6654,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C20" s="9" t="n">
         <f aca="false">Kosten!B18</f>
@@ -6640,7 +6663,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="33" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B21" s="34"/>
       <c r="C21" s="35" t="n">
@@ -6650,7 +6673,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C22" s="9" t="n">
         <f aca="false">Perioden!G8</f>

</xml_diff>